<commit_message>
feat(enemy-mechanics-parity): 召唤代数封顶 + 占用上限
SummonArchetypeId 可以指向另一个同样带召唤字段的原型 = 跨帧指数增殖，
一分钟吃干单位容量；崩起来看着像"关卡莫名其妙停止推进"（导演刷怪全失败），很难查。

两道闸：
- SpawnRequest.Generation + BehaviorArchetype.SummonMaxGeneration
  （判据「本单位代数 < 此值才允许召唤」；1=只有原生能召；0/负按 1 处理）
- SimConst.MaxSpawnGeneration=3：无论怎么配都越不过的硬顶，兜底红线不是平衡旋钮

热更层的召唤与召唤物死亡分裂也走同一套代数，分裂预算算错时内核硬顶仍兜得住。

光有代数封顶不够：实测封顶=2 时代数确实收敛，但"浅而快"的循环照样在 20 秒内
涨到 245/256 吃光导演的槽位。所以再加占用上限 75%，加完同一配置停在 191/256。

Generation 一并进快照，验收能直接看出"第几代"而不是靠数数量猜。
EnemyMechanicsParitySmokeReport 新增 ⑦（原型召唤它自己的最恶劣配置）；仓内 smoke 17/17 PASS。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/cell/#BehaviorArchetype-行为原型.xlsx
+++ b/Configs/GameConfig/Datas/cell/#BehaviorArchetype-行为原型.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD23"/>
+  <dimension ref="A1:AE23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -567,6 +567,11 @@
           <t>summonHealth</t>
         </is>
       </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>summonMaxGeneration</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -719,6 +724,11 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -869,6 +879,11 @@
       <c r="AD3" t="inlineStr">
         <is>
           <t>召唤物生命,0=取宿主生命的1成</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>这支血统最多召到第几代,1=只有原生能召</t>
         </is>
       </c>
     </row>
@@ -965,6 +980,9 @@
       <c r="AD4" t="n">
         <v>0</v>
       </c>
+      <c r="AE4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr"/>
@@ -1057,6 +1075,9 @@
         <v>0</v>
       </c>
       <c r="AD5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1153,6 +1174,9 @@
       <c r="AD6" t="n">
         <v>0</v>
       </c>
+      <c r="AE6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
@@ -1247,6 +1271,9 @@
       <c r="AD7" t="n">
         <v>0</v>
       </c>
+      <c r="AE7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr"/>
@@ -1341,6 +1368,9 @@
       <c r="AD8" t="n">
         <v>0</v>
       </c>
+      <c r="AE8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
@@ -1435,6 +1465,9 @@
       <c r="AD9" t="n">
         <v>0</v>
       </c>
+      <c r="AE9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
@@ -1529,6 +1562,9 @@
       <c r="AD10" t="n">
         <v>0</v>
       </c>
+      <c r="AE10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
@@ -1623,6 +1659,9 @@
       <c r="AD11" t="n">
         <v>0</v>
       </c>
+      <c r="AE11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
@@ -1717,6 +1756,9 @@
       <c r="AD12" t="n">
         <v>0</v>
       </c>
+      <c r="AE12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
@@ -1811,6 +1853,9 @@
       <c r="AD13" t="n">
         <v>0</v>
       </c>
+      <c r="AE13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
@@ -1905,6 +1950,9 @@
       <c r="AD14" t="n">
         <v>0</v>
       </c>
+      <c r="AE14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
@@ -1999,6 +2047,9 @@
       <c r="AD15" t="n">
         <v>0</v>
       </c>
+      <c r="AE15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
@@ -2093,6 +2144,9 @@
       <c r="AD16" t="n">
         <v>0</v>
       </c>
+      <c r="AE16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
@@ -2187,6 +2241,9 @@
       <c r="AD17" t="n">
         <v>0</v>
       </c>
+      <c r="AE17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
@@ -2281,6 +2338,9 @@
       <c r="AD18" t="n">
         <v>0</v>
       </c>
+      <c r="AE18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
@@ -2375,6 +2435,9 @@
       <c r="AD19" t="n">
         <v>0</v>
       </c>
+      <c r="AE19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
@@ -2469,6 +2532,9 @@
       <c r="AD20" t="n">
         <v>0</v>
       </c>
+      <c r="AE20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
@@ -2563,6 +2629,9 @@
       <c r="AD21" t="n">
         <v>0</v>
       </c>
+      <c r="AE21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
@@ -2657,6 +2726,9 @@
       <c r="AD22" t="n">
         <v>0</v>
       </c>
+      <c r="AE22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
@@ -2751,6 +2823,9 @@
       <c r="AD23" t="n">
         <v>8</v>
       </c>
+      <c r="AE23" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>